<commit_message>
Auto update dashboard and allocation
</commit_message>
<xml_diff>
--- a/ETF_Allocation_Model.xlsx
+++ b/ETF_Allocation_Model.xlsx
@@ -486,7 +486,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>73.09999999999999</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -609,7 +609,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>71.2</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -650,7 +650,7 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>75.8</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>63.8</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -732,7 +732,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>81.2</v>
+        <v>81.40000000000001</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Auto update ETF intelligence data
</commit_message>
<xml_diff>
--- a/ETF_Allocation_Model.xlsx
+++ b/ETF_Allocation_Model.xlsx
@@ -486,7 +486,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>71.90000000000001</v>
+        <v>72.7</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -501,7 +501,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Monitorare secondo score e trend.</t>
+          <t>Monitorare secondo score, trend e rischio.</t>
         </is>
       </c>
     </row>
@@ -527,7 +527,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>71.90000000000001</v>
+        <v>71.5</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -568,7 +568,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>81.90000000000001</v>
+        <v>82</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -583,7 +583,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Monitorare secondo score e trend.</t>
+          <t>Monitorare secondo score, trend e rischio.</t>
         </is>
       </c>
     </row>
@@ -609,7 +609,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>70</v>
+        <v>69.5</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -624,7 +624,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Monitorare secondo score e trend.</t>
+          <t>Monitorare secondo score, trend e rischio.</t>
         </is>
       </c>
     </row>
@@ -650,7 +650,7 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>75.8</v>
+        <v>76</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -665,7 +665,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Tema strutturale forte, ma rischio euforia/concentrazione elevato.</t>
+          <t>Tema strutturale forte, ma con rischio euforia e concentrazione.</t>
         </is>
       </c>
     </row>
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>64.3</v>
+        <v>62.2</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -706,7 +706,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Monitorare secondo score e trend.</t>
+          <t>Monitorare secondo score, trend e rischio.</t>
         </is>
       </c>
     </row>
@@ -732,11 +732,11 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>77.2</v>
+        <v>61.3</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Accumulate Carefully</t>
+          <t>Hold / Monitor</t>
         </is>
       </c>
       <c r="G8" t="n">
@@ -747,7 +747,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Utile come protezione macro/geopolitica.</t>
+          <t>Utile come protezione macro/geopolitica. Prezzo sotto media 200: trend non ancora convincente.</t>
         </is>
       </c>
     </row>
@@ -773,7 +773,7 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>35.9</v>
+        <v>38.9</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -788,7 +788,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Componente difensiva, utile per bilanciare rischio equity.</t>
+          <t>Componente difensiva utile per bilanciare il rischio equity. Prezzo sotto media 200: trend non ancora convincente.</t>
         </is>
       </c>
     </row>
@@ -803,7 +803,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -845,10 +845,22 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>Ultimo aggiornamento</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>09/06/2026 09:44</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
           <t>Nota</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>Allocazione indicativa, non consulenza finanziaria personalizzata</t>
         </is>

</xml_diff>

<commit_message>
Auto update ETF data
</commit_message>
<xml_diff>
--- a/ETF_Allocation_Model.xlsx
+++ b/ETF_Allocation_Model.xlsx
@@ -486,7 +486,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>72.7</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -609,7 +609,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>69.5</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -732,7 +732,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>61.3</v>
+        <v>61.2</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -850,7 +850,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>09/06/2026 09:44</t>
+          <t>09/06/2026 11:21</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Apply AlphaForge patch: alpha_forge_v2_core_patch.zip
</commit_message>
<xml_diff>
--- a/ETF_Allocation_Model.xlsx
+++ b/ETF_Allocation_Model.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -440,25 +440,35 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>Peso Target %</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Importo su 1000 EUR</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>Score Finale</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Stato</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Peso Target %</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Importo su 1000 EUR</t>
-        </is>
-      </c>
       <c r="I1" t="inlineStr">
+        <is>
+          <t>Volatilità %</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Max Drawdown %</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
         <is>
           <t>Note AI</t>
         </is>
@@ -472,7 +482,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>iShares Core MSCI Emerging Markets IMI UCITS ETF</t>
+          <t>iShares Core MSCI EM IMI UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -482,38 +492,44 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Emerging Markets</t>
+          <t>Mercati emergenti</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>72.90000000000001</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Accumulate Carefully</t>
-        </is>
+        <v>18.33</v>
+      </c>
+      <c r="F2" t="n">
+        <v>183.3</v>
       </c>
       <c r="G2" t="n">
-        <v>32.5</v>
-      </c>
-      <c r="H2" t="n">
-        <v>325</v>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Monitorare secondo score, trend e rischio.</t>
+        <v>79.3</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Buy Watchlist</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>16.01</v>
+      </c>
+      <c r="J2" t="n">
+        <v>-19.17</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>ETF forte e in trend favorevole; valutare solo con coerenza di portafoglio.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>VWCE.MI</t>
+          <t>VWCE.DE</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Vanguard FTSE All-World UCITS ETF</t>
+          <t>Vanguard FTSE All-World UCITS ETF USD Accumulation</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -523,272 +539,451 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Global Equity</t>
+          <t>Azionario globale</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>71.5</v>
-      </c>
-      <c r="F3" t="inlineStr">
+        <v>18.33</v>
+      </c>
+      <c r="F3" t="n">
+        <v>183.3</v>
+      </c>
+      <c r="G3" t="n">
+        <v>76.40000000000001</v>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>Accumulate Carefully</t>
         </is>
       </c>
-      <c r="G3" t="n">
-        <v>32.5</v>
-      </c>
-      <c r="H3" t="n">
-        <v>325</v>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Buona base core di lungo periodo.</t>
+      <c r="I3" t="n">
+        <v>12.86</v>
+      </c>
+      <c r="J3" t="n">
+        <v>-21.07</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Da monitorare: non è un segnale automatico di acquisto.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>XDEV.MI</t>
+          <t>SWDA.MI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Xtrackers MSCI World Value UCITS ETF</t>
+          <t>iShares Core MSCI World UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Factor</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Value</t>
+          <t>Azionario globale sviluppato</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>82</v>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Buy Watchlist</t>
-        </is>
+        <v>18.33</v>
+      </c>
+      <c r="F4" t="n">
+        <v>183.3</v>
       </c>
       <c r="G4" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="H4" t="n">
-        <v>75</v>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Monitorare secondo score, trend e rischio.</t>
+        <v>75.5</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Accumulate Carefully</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>13.13</v>
+      </c>
+      <c r="J4" t="n">
+        <v>-21.63</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Da monitorare: non è un segnale automatico di acquisto.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>IWQU.MI</t>
+          <t>MVOL.MI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>iShares MSCI World Quality Factor UCITS ETF</t>
+          <t>iShares Edge MSCI World Minimum Volatility UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Factor</t>
+          <t>Defensive</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Quality</t>
+          <t>Min volatility</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>69.59999999999999</v>
-      </c>
-      <c r="F5" t="inlineStr">
+        <v>6.67</v>
+      </c>
+      <c r="F5" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="G5" t="n">
+        <v>68.3</v>
+      </c>
+      <c r="H5" t="inlineStr">
         <is>
           <t>Accumulate Carefully</t>
         </is>
       </c>
-      <c r="G5" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="H5" t="n">
-        <v>75</v>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Monitorare secondo score, trend e rischio.</t>
+      <c r="I5" t="n">
+        <v>9.550000000000001</v>
+      </c>
+      <c r="J5" t="n">
+        <v>-12.85</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Strumento utile per bilanciare volatilità e rischio macro.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>XAIX.MI</t>
+          <t>SGLD.MI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Xtrackers Artificial Intelligence &amp; Big Data UCITS ETF</t>
+          <t>Invesco Physical Gold ETC</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Thematic</t>
+          <t>Defensive</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Artificial Intelligence</t>
+          <t>Oro</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>76</v>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Accumulate Carefully</t>
-        </is>
+        <v>6.67</v>
+      </c>
+      <c r="F6" t="n">
+        <v>66.7</v>
       </c>
       <c r="G6" t="n">
-        <v>5</v>
-      </c>
-      <c r="H6" t="n">
-        <v>50</v>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Tema strutturale forte, ma con rischio euforia e concentrazione.</t>
+        <v>55.5</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Hold / Monitor</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>17.78</v>
+      </c>
+      <c r="J6" t="n">
+        <v>-17.4</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Strumento utile per bilanciare volatilità e rischio macro.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ISPY.MI</t>
+          <t>EUNA.MI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>L&amp;G Cyber Security UCITS ETF</t>
+          <t>iShares Core Global Aggregate Bond</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Thematic</t>
+          <t>Defensive</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Cybersecurity</t>
+          <t>Obbligazionario globale</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>62.2</v>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Hold / Monitor</t>
-        </is>
+        <v>6.67</v>
+      </c>
+      <c r="F7" t="n">
+        <v>66.7</v>
       </c>
       <c r="G7" t="n">
-        <v>5</v>
-      </c>
-      <c r="H7" t="n">
-        <v>50</v>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>Monitorare secondo score, trend e rischio.</t>
+        <v>28.6</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Avoid for Now</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Strumento utile per bilanciare volatilità e rischio macro.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SGLD.MI</t>
+          <t>XDEV.MI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Invesco Physical Gold ETC</t>
+          <t>Xtrackers MSCI World Value UCITS ETF 1C</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Defensive</t>
+          <t>Factor</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Gold</t>
+          <t>Value globale</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>61.2</v>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Hold / Monitor</t>
-        </is>
+        <v>7.5</v>
+      </c>
+      <c r="F8" t="n">
+        <v>75</v>
       </c>
       <c r="G8" t="n">
-        <v>5</v>
-      </c>
-      <c r="H8" t="n">
-        <v>50</v>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>Utile come protezione macro/geopolitica. Prezzo sotto media 200: trend non ancora convincente.</t>
+        <v>79.2</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Accumulate Carefully</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>13.61</v>
+      </c>
+      <c r="J8" t="n">
+        <v>-17.8</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>ETF interessante ma ingresso non ideale: meglio attendere pullback o conferma.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>AGGH.MI</t>
+          <t>IWQU.MI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>iShares Core Global Aggregate Bond UCITS ETF</t>
+          <t>iShares Edge MSCI World Quality Factor UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Defensive</t>
+          <t>Factor</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Global Bonds</t>
+          <t>Quality globale</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>38.9</v>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Avoid for Now</t>
-        </is>
+        <v>7.5</v>
+      </c>
+      <c r="F9" t="n">
+        <v>75</v>
       </c>
       <c r="G9" t="n">
-        <v>5</v>
-      </c>
-      <c r="H9" t="n">
-        <v>50</v>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>Componente difensiva utile per bilanciare il rischio equity. Prezzo sotto media 200: trend non ancora convincente.</t>
+        <v>72.8</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Accumulate Carefully</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>12.86</v>
+      </c>
+      <c r="J9" t="n">
+        <v>-20.6</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Da monitorare: non è un segnale automatico di acquisto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>RBOT.MI</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>iShares Automation &amp; Robotics UCITS ETF USD (Acc)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Thematic</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Robotica e automazione</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>3.33</v>
+      </c>
+      <c r="F10" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="G10" t="n">
+        <v>68.90000000000001</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Accumulate Carefully</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>21.32</v>
+      </c>
+      <c r="J10" t="n">
+        <v>-29.37</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Da monitorare: non è un segnale automatico di acquisto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>INRG.MI</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>iShares Global Clean Energy Transition UCITS ETF USD (Dist)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Thematic</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Energia pulita</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>3.33</v>
+      </c>
+      <c r="F11" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="G11" t="n">
+        <v>64.3</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Hold / Monitor</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>23.17</v>
+      </c>
+      <c r="J11" t="n">
+        <v>-44.26</v>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Rischio elevato: usare solo come quota satellite e con size ridotta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>SMH</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>VanEck Semiconductor ETF</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Thematic</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Semiconduttori</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>3.33</v>
+      </c>
+      <c r="F12" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="G12" t="n">
+        <v>61.9</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Hold / Monitor</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>34.92</v>
+      </c>
+      <c r="J12" t="n">
+        <v>-35.74</v>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Rischio elevato: usare solo come quota satellite e con size ridotta.</t>
         </is>
       </c>
     </row>
@@ -803,7 +998,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -833,36 +1028,42 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Importo simulato</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>1000 EUR</t>
-        </is>
+          <t>ETF analizzati</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ultimo aggiornamento</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>09/06/2026 11:21</t>
-        </is>
+          <t>ETF in allocazione</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>Score medio</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>65.92</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
           <t>Nota</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Allocazione indicativa, non consulenza finanziaria personalizzata</t>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Allocazione informativa su 1000 EUR, non consulenza personalizzata.</t>
         </is>
       </c>
     </row>

</xml_diff>